<commit_message>
STRY0067504: connection settings via system properties, no Outbound REST Message record
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/docs/rm_story_drafts_ready.xlsx
+++ b/docs/rm_story_drafts_ready.xlsx
@@ -508,11 +508,11 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Create Outbound REST Message for AdaptiveWork (Clarizen) API</t>
+          <t>Configure AdaptiveWork API connection settings (Dev, Test, Prod)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -521,21 +521,20 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Connection is proven in Dev. This story closes it out and makes it repeatable in Test and Prod.
+          <t>No Outbound REST Message record is needed: every Data Source and script calls the API directly (sn_ws.RESTMessageV2) and reads the address and key from system properties. This is how the working 'Adaptive Projects - API' Data Source runs in Dev.
 This story is complete when:
 - System properties exist: x_mig.adaptive.url (string) = https://api2.clarizen.com/v2.0/services; x_mig.adaptive.key (password2). No key appears in any script.
-- Header used by every call: Authorization: ApiKey &lt;x_mig.adaptive.key&gt;; Content-Type: application/json.
-- Test 1: POST {url}/data/query with {"q":"SELECT Name FROM Project","paging":{"from":0,"limit":2}} returns 200 and two projects.
+- Test 1 (Scripts - Background): POST {url}/data/query with {"q":"SELECT Name FROM Project","paging":{"from":0,"limit":2}} and header Authorization: ApiKey &lt;key&gt; returns 200 and two projects.
 - Test 2: GET {url}/metadata/describeEntities?typeNames=Project returns 200 (GET - POST returns 404).
-- The key is switched to the svc_sn_migration service account key when issued (property value only).
-- The same properties are created in Test and Prod (values are entered per instance).</t>
+- The key value is switched to the svc_sn_migration service account key when issued.
+- The same properties are created in Test and Prod (values are entered per instance; they do not move with code), and Test 1 passes in each.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Connection is proven in Dev. This story closes it out and makes it repeatable in Test and Prod.&lt;/p&gt;
+          <t>&lt;p&gt;No Outbound REST Message record is needed: every Data Source and script calls the API directly (sn_ws.RESTMessageV2) and reads the address and key from system properties. This is how the working &amp;#x27;Adaptive Projects - API&amp;#x27; Data Source runs in Dev.&lt;/p&gt;
 &lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;System properties exist: x_mig.adaptive.url (string) = https://api2.clarizen.com/v2.0/services; x_mig.adaptive.key (password2). No key appears in any script.&lt;/li&gt;&lt;li&gt;Header used by every call: Authorization: ApiKey &amp;lt;x_mig.adaptive.key&amp;gt;; Content-Type: application/json.&lt;/li&gt;&lt;li&gt;Test 1: POST {url}/data/query with {&amp;quot;q&amp;quot;:&amp;quot;SELECT Name FROM Project&amp;quot;,&amp;quot;paging&amp;quot;:{&amp;quot;from&amp;quot;:0,&amp;quot;limit&amp;quot;:2}} returns 200 and two projects.&lt;/li&gt;&lt;li&gt;Test 2: GET {url}/metadata/describeEntities?typeNames=Project returns 200 (GET - POST returns 404).&lt;/li&gt;&lt;li&gt;The key is switched to the svc_sn_migration service account key when issued (property value only).&lt;/li&gt;&lt;li&gt;The same properties are created in Test and Prod (values are entered per instance).&lt;/li&gt;&lt;/ul&gt;</t>
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;System properties exist: x_mig.adaptive.url (string) = https://api2.clarizen.com/v2.0/services; x_mig.adaptive.key (password2). No key appears in any script.&lt;/li&gt;&lt;li&gt;Test 1 (Scripts - Background): POST {url}/data/query with {&amp;quot;q&amp;quot;:&amp;quot;SELECT Name FROM Project&amp;quot;,&amp;quot;paging&amp;quot;:{&amp;quot;from&amp;quot;:0,&amp;quot;limit&amp;quot;:2}} and header Authorization: ApiKey &amp;lt;key&amp;gt; returns 200 and two projects.&lt;/li&gt;&lt;li&gt;Test 2: GET {url}/metadata/describeEntities?typeNames=Project returns 200 (GET - POST returns 404).&lt;/li&gt;&lt;li&gt;The key value is switched to the svc_sn_migration service account key when issued.&lt;/li&gt;&lt;li&gt;The same properties are created in Test and Prod (values are entered per instance; they do not move with code), and Test 1 passes in each.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -874,7 +873,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Staging table is u_import_asana_hr_project_portfolio (story says u_imp_asana_hr_portfolio). Project GID = 1208928603143252 (HR Project Portfolio 2026; workspace 5286451799521 is not the project). Use a Data Source 'Custom (Load by Script)' instead of a Scheduled Job, so the transform map runs on the loaded rows: servicenow/asana_data_source.js (MODE 'projects'; MODE 'tasks' for the work plan) already does AC 2-5. Add assignee.name and gid to opt_fields. Token is in property x_mig.asana.token (password2), proven 200 in Dev.</t>
+          <t>AC 1: no Outbound REST Message record is needed - the Data Source script calls Asana directly and reads the token from property x_mig.asana.token (same as Adaptive). Staging table is u_import_asana_hr_project_portfolio (story says u_imp_asana_hr_portfolio). Project GID = 1208928603143252 (HR Project Portfolio 2026; workspace 5286451799521 is not the project). Use a Data Source 'Custom (Load by Script)' instead of a Scheduled Job, so the transform map runs on the loaded rows: servicenow/asana_data_source.js (MODE 'projects'; MODE 'tasks' for the work plan) already does AC 2-5. Add assignee.name and gid to opt_fields. Token is in property x_mig.asana.token (password2), proven 200 in Dev.</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1102,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Close out connection (Dev, then Test/Prod properties)</t>
+          <t>Connection settings (system properties) in Dev, Test, Prod - no REST Message record</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify the Draft stories: short steps, detail moved into ready-to-paste scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/docs/rm_story_drafts_ready.xlsx
+++ b/docs/rm_story_drafts_ready.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Drafts - assign" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="In flight - fixes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Drafts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="In-flight fixes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Build order" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -446,16 +446,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="100" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,30 +465,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Assign now?</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Short description</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Points</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Depends on</t>
+          <t>Acceptance criteria</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Acceptance criteria</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Acceptance criteria (HTML - paste into ServiceNow)</t>
         </is>
@@ -501,40 +495,32 @@
           <t>STRY0067504</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Set up the Adaptive and Asana API connection settings</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Configure AdaptiveWork API connection settings (Dev, Test, Prod)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>This story is complete when:
+- These system properties exist in Dev, Test and Prod: x_mig.adaptive.url, x_mig.adaptive.key (password2), x_mig.asana.token (password2), x_mig.asana.project_gid.
+- The keys are the svc_sn_migration service account keys.
+- servicenow/test_connection.js, run in Scripts - Background, shows Status: 200 for Adaptive and Asana in each instance.
+- No Outbound REST Message is needed.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No Outbound REST Message record is needed: every Data Source and script calls the API directly (sn_ws.RESTMessageV2) and reads the address and key from system properties. This is how the working 'Adaptive Projects - API' Data Source runs in Dev.
-This story is complete when:
-- System properties exist: x_mig.adaptive.url (string) = https://api2.clarizen.com/v2.0/services; x_mig.adaptive.key (password2). No key appears in any script.
-- Test 1 (Scripts - Background): POST {url}/data/query with {"q":"SELECT Name FROM Project","paging":{"from":0,"limit":2}} and header Authorization: ApiKey &lt;key&gt; returns 200 and two projects.
-- Test 2: GET {url}/metadata/describeEntities?typeNames=Project returns 200 (GET - POST returns 404).
-- The key value is switched to the svc_sn_migration service account key when issued.
-- The same properties are created in Test and Prod (values are entered per instance; they do not move with code), and Test 1 passes in each.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;No Outbound REST Message record is needed: every Data Source and script calls the API directly (sn_ws.RESTMessageV2) and reads the address and key from system properties. This is how the working &amp;#x27;Adaptive Projects - API&amp;#x27; Data Source runs in Dev.&lt;/p&gt;
-&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;System properties exist: x_mig.adaptive.url (string) = https://api2.clarizen.com/v2.0/services; x_mig.adaptive.key (password2). No key appears in any script.&lt;/li&gt;&lt;li&gt;Test 1 (Scripts - Background): POST {url}/data/query with {&amp;quot;q&amp;quot;:&amp;quot;SELECT Name FROM Project&amp;quot;,&amp;quot;paging&amp;quot;:{&amp;quot;from&amp;quot;:0,&amp;quot;limit&amp;quot;:2}} and header Authorization: ApiKey &amp;lt;key&amp;gt; returns 200 and two projects.&lt;/li&gt;&lt;li&gt;Test 2: GET {url}/metadata/describeEntities?typeNames=Project returns 200 (GET - POST returns 404).&lt;/li&gt;&lt;li&gt;The key value is switched to the svc_sn_migration service account key when issued.&lt;/li&gt;&lt;li&gt;The same properties are created in Test and Prod (values are entered per instance; they do not move with code), and Test 1 passes in each.&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;These system properties exist in Dev, Test and Prod: x_mig.adaptive.url, x_mig.adaptive.key (password2), x_mig.asana.token (password2), x_mig.asana.project_gid.&lt;/li&gt;&lt;li&gt;The keys are the svc_sn_migration service account keys.&lt;/li&gt;&lt;li&gt;servicenow/test_connection.js, run in Scripts - Background, shows Status: 200 for Adaptive and Asana in each instance.&lt;/li&gt;&lt;li&gt;No Outbound REST Message is needed.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -544,52 +530,33 @@
           <t>STRY0067506</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Create the Adaptive Data Sources for project-related records</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Create API Data Sources and Staging Tables for AdaptiveWork Entities</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>STRY0067504; projects loaded (STRY0066697)</t>
+          <t>This story is complete when:
+- servicenow/discovery_background_script.js has been run once, and its output is attached to this story.
+- One Data Source (Type: Custom (Load by Script)) exists for each: Tasks, Milestones, Risks, Issues, Lessons Learned, Resources, Time.
+- Each uses servicenow/adaptive_related_data_source.js. Only the settings block at the top changes, using the names from the Discovery output.
+- Each import table has the columns Correlation ID, Parent Correlation ID and Project Correlation ID.
+- Load All Records runs with no errors for the pilot projects.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source 'Adaptive Projects - API' -&gt; u_import_adaptive_projects -&gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = "ADAPTIVE:" + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or "ASANA:" + Asana gid. Scripts: repo folder servicenow/.
-No Scheduled Data Imports: each Data Source is Type 'Custom (Load by Script)' and is run by hand in build order (scheduling adds nothing for a one-time migration).
-This story is complete when:
-- Discovery: servicenow/discovery_background_script.js is run in Scripts - Background and its output is attached to this story. It lists the real Adaptive entity and field names; every [CONFIRM] below is filled from it before building that Data Source.
-- Each staging table below has String(100) columns Correlation ID, Parent Correlation ID, Project Correlation ID (added like Correlation ID on u_import_adaptive_projects).
-- Each Data Source uses servicenow/adaptive_related_data_source.js with only its CONFIG block changed (ENTITY, PROJECT_FIELD, MAP of column label -&gt; Adaptive field). The script loads records only for projects already in pm_project with an ADAPTIVE: correlation_id, follows paging, and flattens references ({"id":"/State/Active"} -&gt; Active; dates -&gt; yyyy-MM-dd).
-- Load All Records on each completes with no import-log errors, and the log line 'rows loaded: N (for M projects)' matches Adaptive for the pilot projects.
-- Demands: not built until the Demand vs Project rule is confirmed (STRY0066695).
-Data Source | Staging table | ENTITY | PROJECT_FIELD | Used by
-Adaptive Projects - API (done) | u_import_adaptive_projects | Project | - | STRY0066697, STRY0066701
-Adaptive Tasks - API | u_import_adaptive_project_tasks | Task | Project | STRY0066699
-Adaptive Milestones - API | u_import_adaptive_project_tasks | Milestone | Project | STRY0066699 (Milestone = '=true')
-Adaptive Risks - API | u_import_adaptive_risks | [CONFIRM] Risk | [CONFIRM] | STRY0066718
-Adaptive Issues - API | u_import_adaptive_issues | [CONFIRM] Issue | [CONFIRM] | STRY0066715
-Adaptive Lessons - API | [new] u_import_adaptive_lessons | C_PMOLessonsLearned | C_RelatedWorkItem | STRY0067099
-Adaptive Resources - API | [new] u_import_adaptive_resources | [CONFIRM] resource link entity | [CONFIRM] | STRY0066702
-Adaptive Time - API | [new] u_import_adaptive_time | [CONFIRM] timesheet entity | [CONFIRM] | STRY0066702</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source &amp;#x27;Adaptive Projects - API&amp;#x27; -&amp;gt; u_import_adaptive_projects -&amp;gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts: repo folder servicenow/.&lt;/p&gt;
-&lt;p&gt;No Scheduled Data Imports: each Data Source is Type &amp;#x27;Custom (Load by Script)&amp;#x27; and is run by hand in build order (scheduling adds nothing for a one-time migration).&lt;/p&gt;
-&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Discovery: servicenow/discovery_background_script.js is run in Scripts - Background and its output is attached to this story. It lists the real Adaptive entity and field names; every [CONFIRM] below is filled from it before building that Data Source.&lt;/li&gt;&lt;li&gt;Each staging table below has String(100) columns Correlation ID, Parent Correlation ID, Project Correlation ID (added like Correlation ID on u_import_adaptive_projects).&lt;/li&gt;&lt;li&gt;Each Data Source uses servicenow/adaptive_related_data_source.js with only its CONFIG block changed (ENTITY, PROJECT_FIELD, MAP of column label -&amp;gt; Adaptive field). The script loads records only for projects already in pm_project with an ADAPTIVE: correlation_id, follows paging, and flattens references ({&amp;quot;id&amp;quot;:&amp;quot;/State/Active&amp;quot;} -&amp;gt; Active; dates -&amp;gt; yyyy-MM-dd).&lt;/li&gt;&lt;li&gt;Load All Records on each completes with no import-log errors, and the log line &amp;#x27;rows loaded: N (for M projects)&amp;#x27; matches Adaptive for the pilot projects.&lt;/li&gt;&lt;li&gt;Demands: not built until the Demand vs Project rule is confirmed (STRY0066695).&lt;/li&gt;&lt;/ul&gt;
-&lt;table style="width: 100%;"&gt;&lt;thead&gt;&lt;tr&gt;&lt;td&gt;&lt;strong&gt;Data Source&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;Staging table&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;ENTITY&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;PROJECT_FIELD&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;Used by&lt;/strong&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Adaptive Projects - API (done)&lt;/td&gt;&lt;td&gt;u_import_adaptive_projects&lt;/td&gt;&lt;td&gt;Project&lt;/td&gt;&lt;td&gt;-&lt;/td&gt;&lt;td&gt;STRY0066697, STRY0066701&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Tasks - API&lt;/td&gt;&lt;td&gt;u_import_adaptive_project_tasks&lt;/td&gt;&lt;td&gt;Task&lt;/td&gt;&lt;td&gt;Project&lt;/td&gt;&lt;td&gt;STRY0066699&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Milestones - API&lt;/td&gt;&lt;td&gt;u_import_adaptive_project_tasks&lt;/td&gt;&lt;td&gt;Milestone&lt;/td&gt;&lt;td&gt;Project&lt;/td&gt;&lt;td&gt;STRY0066699 (Milestone = &amp;#x27;=true&amp;#x27;)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Risks - API&lt;/td&gt;&lt;td&gt;u_import_adaptive_risks&lt;/td&gt;&lt;td&gt;[CONFIRM] Risk&lt;/td&gt;&lt;td&gt;[CONFIRM]&lt;/td&gt;&lt;td&gt;STRY0066718&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Issues - API&lt;/td&gt;&lt;td&gt;u_import_adaptive_issues&lt;/td&gt;&lt;td&gt;[CONFIRM] Issue&lt;/td&gt;&lt;td&gt;[CONFIRM]&lt;/td&gt;&lt;td&gt;STRY0066715&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Lessons - API&lt;/td&gt;&lt;td&gt;[new] u_import_adaptive_lessons&lt;/td&gt;&lt;td&gt;C_PMOLessonsLearned&lt;/td&gt;&lt;td&gt;C_RelatedWorkItem&lt;/td&gt;&lt;td&gt;STRY0067099&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Resources - API&lt;/td&gt;&lt;td&gt;[new] u_import_adaptive_resources&lt;/td&gt;&lt;td&gt;[CONFIRM] resource link entity&lt;/td&gt;&lt;td&gt;[CONFIRM]&lt;/td&gt;&lt;td&gt;STRY0066702&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Adaptive Time - API&lt;/td&gt;&lt;td&gt;[new] u_import_adaptive_time&lt;/td&gt;&lt;td&gt;[CONFIRM] timesheet entity&lt;/td&gt;&lt;td&gt;[CONFIRM]&lt;/td&gt;&lt;td&gt;STRY0066702&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;servicenow/discovery_background_script.js has been run once, and its output is attached to this story.&lt;/li&gt;&lt;li&gt;One Data Source (Type: Custom (Load by Script)) exists for each: Tasks, Milestones, Risks, Issues, Lessons Learned, Resources, Time.&lt;/li&gt;&lt;li&gt;Each uses servicenow/adaptive_related_data_source.js. Only the settings block at the top changes, using the names from the Discovery output.&lt;/li&gt;&lt;li&gt;Each import table has the columns Correlation ID, Parent Correlation ID and Project Correlation ID.&lt;/li&gt;&lt;li&gt;Load All Records runs with no errors for the pilot projects.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -599,76 +566,32 @@
           <t>STRY0066701</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Create status reports from Adaptive project health</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Create Transform Map: Migrate Adaptive Health to Status Reports (project_status)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>STRY0066697</t>
+          <t>This story is complete when:
+- A new transform map turns the Adaptive Projects import into status reports (project_status), set up as described at the top of servicenow/status_report_transform.js.
+- Health colours: On Target / On Plan = Green, Needs Attention = Yellow, In Trouble = Red.
+- Update Notes go into the status report comments.
+- Each pilot project has one status report, and running it again adds no new ones.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source 'Adaptive Projects - API' -&gt; u_import_adaptive_projects -&gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = "ADAPTIVE:" + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or "ASANA:" + Asana gid. Scripts: repo folder servicenow/.
-Source: Adaptive keeps health on the project (Health, Schedule/Budget/Resource/Scope/Risk Health, Update Notes), already loaded into u_import_adaptive_projects. No extra API call: a second transform map on the same staging table creates one status report per project. Asana: not in scope (HR portfolio items have no status reports).
-This story is complete when:
-- System property x_mig.status_as_on (string, yyyy-MM-dd) = the migration date. A fixed date makes reruns update the same report.
-- Transform map 'Import Adaptive Status Reports': u_import_adaptive_projects -&gt; project_status, Order 200 (project map Order 100). Run Transform selects both maps.
-- Field map [Script] -&gt; project, Coalesce = true: sys_id of the pm_project whose correlation_id = source.u_correlation_id (skip row if none).
-- Field map [Script] -&gt; as_on, Coalesce = true: gs.getProperty('x_mig.status_as_on').
-- onBefore below sets the 5 health fields (value table below) and comments; a project with no health values gets no report. Choice action on the health fields = Reject.
-- Staging column names used: u_health, u_schedule_health, u_budget_health, u_resource_health, u_scope_health, u_risk_health, u_update_notes (dev confirms on the table's Columns tab).
-- Done when each pilot project has 1 status report matching Adaptive's colours, and a rerun adds none.
-(function runTransformScript(source, map, log, target) {
-    var rag = { 'on target': 'green', 'on plan': 'green', 'needs attention': 'yellow', 'in trouble': 'red' };
-    function c(v) { return rag[(v + '').toLowerCase().trim()] || ''; }
-    target.overall_health = c(source.u_health);
-    target.schedule  = c(source.u_schedule_health);
-    target.cost      = c(source.u_budget_health);
-    target.resources = c(source.u_resource_health);
-    target.scope     = c(source.u_scope_health);
-    if (!target.overall_health &amp;&amp; !target.schedule &amp;&amp; !target.cost &amp;&amp; !target.resources &amp;&amp; !target.scope) { ignore = true; return; }
-    var risk = source.u_risk_health + '';
-    var notes = (source.u_update_notes + '').replace(/&lt;[^&gt;]+&gt;/g, ' ').replace(/&amp;nbsp;/g, ' ');
-    target.comments = (risk ? 'Risk health (Adaptive): ' + risk + '\n' : '') + notes;
-})(source, map, log, target);
-Adaptive value | project_status value
-On Target / On Plan | green
-Needs Attention | yellow
-In Trouble | red
-blank | (empty)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source &amp;#x27;Adaptive Projects - API&amp;#x27; -&amp;gt; u_import_adaptive_projects -&amp;gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts: repo folder servicenow/.&lt;/p&gt;
-&lt;p&gt;Source: Adaptive keeps health on the project (Health, Schedule/Budget/Resource/Scope/Risk Health, Update Notes), already loaded into u_import_adaptive_projects. No extra API call: a second transform map on the same staging table creates one status report per project. Asana: not in scope (HR portfolio items have no status reports).&lt;/p&gt;
-&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;System property x_mig.status_as_on (string, yyyy-MM-dd) = the migration date. A fixed date makes reruns update the same report.&lt;/li&gt;&lt;li&gt;Transform map &amp;#x27;Import Adaptive Status Reports&amp;#x27;: u_import_adaptive_projects -&amp;gt; project_status, Order 200 (project map Order 100). Run Transform selects both maps.&lt;/li&gt;&lt;li&gt;Field map [Script] -&amp;gt; project, Coalesce = true: sys_id of the pm_project whose correlation_id = source.u_correlation_id (skip row if none).&lt;/li&gt;&lt;li&gt;Field map [Script] -&amp;gt; as_on, Coalesce = true: gs.getProperty(&amp;#x27;x_mig.status_as_on&amp;#x27;).&lt;/li&gt;&lt;li&gt;onBefore below sets the 5 health fields (value table below) and comments; a project with no health values gets no report. Choice action on the health fields = Reject.&lt;/li&gt;&lt;li&gt;Staging column names used: u_health, u_schedule_health, u_budget_health, u_resource_health, u_scope_health, u_risk_health, u_update_notes (dev confirms on the table&amp;#x27;s Columns tab).&lt;/li&gt;&lt;li&gt;Done when each pilot project has 1 status report matching Adaptive&amp;#x27;s colours, and a rerun adds none.&lt;/li&gt;&lt;/ul&gt;
-&lt;pre&gt;&lt;code&gt;(function runTransformScript(source, map, log, target) {
-    var rag = { &amp;#x27;on target&amp;#x27;: &amp;#x27;green&amp;#x27;, &amp;#x27;on plan&amp;#x27;: &amp;#x27;green&amp;#x27;, &amp;#x27;needs attention&amp;#x27;: &amp;#x27;yellow&amp;#x27;, &amp;#x27;in trouble&amp;#x27;: &amp;#x27;red&amp;#x27; };
-    function c(v) { return rag[(v + &amp;#x27;&amp;#x27;).toLowerCase().trim()] || &amp;#x27;&amp;#x27;; }
-    target.overall_health = c(source.u_health);
-    target.schedule  = c(source.u_schedule_health);
-    target.cost      = c(source.u_budget_health);
-    target.resources = c(source.u_resource_health);
-    target.scope     = c(source.u_scope_health);
-    if (!target.overall_health &amp;amp;&amp;amp; !target.schedule &amp;amp;&amp;amp; !target.cost &amp;amp;&amp;amp; !target.resources &amp;amp;&amp;amp; !target.scope) { ignore = true; return; }
-    var risk = source.u_risk_health + &amp;#x27;&amp;#x27;;
-    var notes = (source.u_update_notes + &amp;#x27;&amp;#x27;).replace(/&amp;lt;[^&amp;gt;]+&amp;gt;/g, &amp;#x27; &amp;#x27;).replace(/&amp;amp;nbsp;/g, &amp;#x27; &amp;#x27;);
-    target.comments = (risk ? &amp;#x27;Risk health (Adaptive): &amp;#x27; + risk + &amp;#x27;\n&amp;#x27; : &amp;#x27;&amp;#x27;) + notes;
-})(source, map, log, target);&lt;/code&gt;&lt;/pre&gt;
-&lt;table style="width: 100%;"&gt;&lt;thead&gt;&lt;tr&gt;&lt;td&gt;&lt;strong&gt;Adaptive value&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;project_status value&lt;/strong&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;On Target / On Plan&lt;/td&gt;&lt;td&gt;green&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Needs Attention&lt;/td&gt;&lt;td&gt;yellow&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;In Trouble&lt;/td&gt;&lt;td&gt;red&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;blank&lt;/td&gt;&lt;td&gt;(empty)&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;A new transform map turns the Adaptive Projects import into status reports (project_status), set up as described at the top of servicenow/status_report_transform.js.&lt;/li&gt;&lt;li&gt;Health colours: On Target / On Plan = Green, Needs Attention = Yellow, In Trouble = Red.&lt;/li&gt;&lt;li&gt;Update Notes go into the status report comments.&lt;/li&gt;&lt;li&gt;Each pilot project has one status report, and running it again adds no new ones.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -678,44 +601,33 @@
           <t>STRY0066702</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Yes (scope as written)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Migrate Adaptive Resource Assignments and Time (actual effort) to Project Tasks</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Add people and hours worked to project tasks (Adaptive)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>8</v>
       </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>STRY0067506 (Resources, Time); STRY0066699</t>
+          <t>This story is complete when:
+- Adaptive resource assignments are loaded: the first person becomes Assigned to; others go into Additional assignee list.
+- Adaptive time is loaded as total hours per task into the task's actual effort.
+- These loads only update existing tasks; they never create new ones. Scripts: servicenow/resources_time_transform.js.
+- Rate models, weekly time cards and resource plans are out of scope.
+- 5 pilot tasks show the same people and hours as Adaptive.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source 'Adaptive Projects - API' -&gt; u_import_adaptive_projects -&gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = "ADAPTIVE:" + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or "ASANA:" + Asana gid. Scripts: repo folder servicenow/.
-Scope: (1) the people on each task, (2) hours already worked per task. NOT in scope unless the BA decides otherwise: rate models, weekly time cards, resource plans/allocations (they create cost and Resource Management records that need fiscal periods, rates and approvals).
-This story is complete when:
-- Resources: transform map u_import_adaptive_resources -&gt; pm_project_task. [Script] -&gt; correlation_id (Coalesce = true) returns source.u_project_correlation_id (the task the person is linked to).
-- Resources onBefore: if no pm_project_task has that correlation_id, ignore = true (this map never creates tasks). First person -&gt; assigned_to; others are added to additional_assignee_list without duplicates. Users match sys_user on email; no match -&gt; log.warn, field left as is.
-- Links on a project (ADAPTIVE:/Project/...) go through a second map on the same staging table -&gt; pm_project (same rules), adding people to the project's additional_assignee_list.
-- Time: the 'Adaptive Time - API' Data Source sums hours per work item and inserts one row per task (Project Correlation ID = the task, Total Hours).
-- Time map u_import_adaptive_time -&gt; pm_project_task, same coalesce and same 'never create' guard; Total Hours -&gt; the task's actual effort field (dev confirms the element name in the pm_project_task dictionary).
-- Asana: no separate feed. Assignee and collaborators come with the Asana work plan (STRY0065275); time only if Discovery shows actual_time_minutes.
-- Done when 5 pilot tasks show the same people and total hours as Adaptive, and a rerun changes nothing.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source &amp;#x27;Adaptive Projects - API&amp;#x27; -&amp;gt; u_import_adaptive_projects -&amp;gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts: repo folder servicenow/.&lt;/p&gt;
-&lt;p&gt;Scope: (1) the people on each task, (2) hours already worked per task. NOT in scope unless the BA decides otherwise: rate models, weekly time cards, resource plans/allocations (they create cost and Resource Management records that need fiscal periods, rates and approvals).&lt;/p&gt;
-&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Resources: transform map u_import_adaptive_resources -&amp;gt; pm_project_task. [Script] -&amp;gt; correlation_id (Coalesce = true) returns source.u_project_correlation_id (the task the person is linked to).&lt;/li&gt;&lt;li&gt;Resources onBefore: if no pm_project_task has that correlation_id, ignore = true (this map never creates tasks). First person -&amp;gt; assigned_to; others are added to additional_assignee_list without duplicates. Users match sys_user on email; no match -&amp;gt; log.warn, field left as is.&lt;/li&gt;&lt;li&gt;Links on a project (ADAPTIVE:/Project/...) go through a second map on the same staging table -&amp;gt; pm_project (same rules), adding people to the project&amp;#x27;s additional_assignee_list.&lt;/li&gt;&lt;li&gt;Time: the &amp;#x27;Adaptive Time - API&amp;#x27; Data Source sums hours per work item and inserts one row per task (Project Correlation ID = the task, Total Hours).&lt;/li&gt;&lt;li&gt;Time map u_import_adaptive_time -&amp;gt; pm_project_task, same coalesce and same &amp;#x27;never create&amp;#x27; guard; Total Hours -&amp;gt; the task&amp;#x27;s actual effort field (dev confirms the element name in the pm_project_task dictionary).&lt;/li&gt;&lt;li&gt;Asana: no separate feed. Assignee and collaborators come with the Asana work plan (STRY0065275); time only if Discovery shows actual_time_minutes.&lt;/li&gt;&lt;li&gt;Done when 5 pilot tasks show the same people and total hours as Adaptive, and a rerun changes nothing.&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Adaptive resource assignments are loaded: the first person becomes Assigned to; others go into Additional assignee list.&lt;/li&gt;&lt;li&gt;Adaptive time is loaded as total hours per task into the task&amp;#x27;s actual effort.&lt;/li&gt;&lt;li&gt;These loads only update existing tasks; they never create new ones. Scripts: servicenow/resources_time_transform.js.&lt;/li&gt;&lt;li&gt;Rate models, weekly time cards and resource plans are out of scope.&lt;/li&gt;&lt;li&gt;5 pilot tasks show the same people and hours as Adaptive.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -725,45 +637,33 @@
           <t>STRY0066723</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Yes (build now, run last)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Migrate Legacy Attachments from Asana and Adaptive via API</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Copy attachments from Asana and Adaptive</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Yes - run last</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>All record loads</t>
+          <t>This story is complete when:
+- servicenow/attachments_fix_script.js is run as a Fix Script after all other loads.
+- It is run first with DRY_RUN = true, and the log reviewed. Then it is run with DRY_RUN = false.
+- Files stored in Google Drive, Box, Dropbox or OneDrive are added to the record as a link in a work note.
+- Running it again does not create duplicate files.
+- 10 spot-checked files open correctly in ServiceNow.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source 'Adaptive Projects - API' -&gt; u_import_adaptive_projects -&gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = "ADAPTIVE:" + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or "ASANA:" + Asana gid. Scripts: repo folder servicenow/.
-Replaces manual download/upload. Script: servicenow/attachments_fix_script.js (Fix Script).
-This story is complete when:
-- Asana: for each migrated record with an ASANA: correlation_id, GET https://app.asana.com/api/1.0/attachments?parent=&lt;gid&gt;&amp;opt_fields=name,host,size,download_url,view_url.
-- Files with host = asana are downloaded from download_url (a short-lived signed link: fetched immediately and WITHOUT the Asana token) and saved with RESTMessageV2.saveResponseBodyAsAttachment(table, sys_id, file name).
-- Files hosted elsewhere (Google Drive, Box, Dropbox, OneDrive) cannot be downloaded: their name and view_url are added as a work note on the record.
-- Adaptive: files linked to each ADAPTIVE: record; the link query and download path are set at the top of the script from the Discovery output (ADAPTIVE_LINK_QUERY, ADAPTIVE_DOWNLOAD) [CONFIRM].
-- Tables: pm_project, pm_project_task, dmn_demand, risk, issue (as loaded).
-- Run 1 with DRY_RUN = true; System Logs (source x_mig.attachments) shows what would be copied. Run 2 with DRY_RUN = false.
-- Rerun-safe: a file with the same name already on the record is skipped. Files over 50 MB are logged for manual copy.
-- Done when the final log line shows failed = 0 (or each failure is listed and resolved) and 10 files are opened successfully in ServiceNow.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Already working in Dev: system properties x_mig.adaptive.url (https://api2.clarizen.com/v2.0/services), x_mig.adaptive.key, x_mig.asana.token, x_mig.asana.project_gid (1208928603143252 = HR Project Portfolio 2026); Data Source &amp;#x27;Adaptive Projects - API&amp;#x27; -&amp;gt; u_import_adaptive_projects -&amp;gt; Import Adaptive Projects Transform Map (PRJ0010675 created). Key rule for every map: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts: repo folder servicenow/.&lt;/p&gt;
-&lt;p&gt;Replaces manual download/upload. Script: servicenow/attachments_fix_script.js (Fix Script).&lt;/p&gt;
-&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Asana: for each migrated record with an ASANA: correlation_id, GET https://app.asana.com/api/1.0/attachments?parent=&amp;lt;gid&amp;gt;&amp;amp;opt_fields=name,host,size,download_url,view_url.&lt;/li&gt;&lt;li&gt;Files with host = asana are downloaded from download_url (a short-lived signed link: fetched immediately and WITHOUT the Asana token) and saved with RESTMessageV2.saveResponseBodyAsAttachment(table, sys_id, file name).&lt;/li&gt;&lt;li&gt;Files hosted elsewhere (Google Drive, Box, Dropbox, OneDrive) cannot be downloaded: their name and view_url are added as a work note on the record.&lt;/li&gt;&lt;li&gt;Adaptive: files linked to each ADAPTIVE: record; the link query and download path are set at the top of the script from the Discovery output (ADAPTIVE_LINK_QUERY, ADAPTIVE_DOWNLOAD) [CONFIRM].&lt;/li&gt;&lt;li&gt;Tables: pm_project, pm_project_task, dmn_demand, risk, issue (as loaded).&lt;/li&gt;&lt;li&gt;Run 1 with DRY_RUN = true; System Logs (source x_mig.attachments) shows what would be copied. Run 2 with DRY_RUN = false.&lt;/li&gt;&lt;li&gt;Rerun-safe: a file with the same name already on the record is skipped. Files over 50 MB are logged for manual copy.&lt;/li&gt;&lt;li&gt;Done when the final log line shows failed = 0 (or each failure is listed and resolved) and 10 files are opened successfully in ServiceNow.&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;servicenow/attachments_fix_script.js is run as a Fix Script after all other loads.&lt;/li&gt;&lt;li&gt;It is run first with DRY_RUN = true, and the log reviewed. Then it is run with DRY_RUN = false.&lt;/li&gt;&lt;li&gt;Files stored in Google Drive, Box, Dropbox or OneDrive are added to the record as a link in a work note.&lt;/li&gt;&lt;li&gt;Running it again does not create duplicate files.&lt;/li&gt;&lt;li&gt;10 spot-checked files open correctly in ServiceNow.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -773,43 +673,29 @@
           <t>STRY0066721</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Create cost plans from Adaptive budgets</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Create Transform Map: Migrate Adaptive Budgets to Cost Plans (cost_plan)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>6</v>
-      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>BA decision: budget source + cost plans vs demand totals</t>
+          <t>This story is complete when:
+- On hold until the BA confirms (1) where budgets live in Adaptive and (2) cost plans or demand budget totals (not both).</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not ready to assign: two answers are needed first, otherwise the dev builds against a guess.
-- Where budgets live in Adaptive: project fields or a budget/expense entity (the Discovery output in STRY0067506 lists the candidates).
-- Cost plans or demand budget totals (STRY0066695) - not both: cost plans roll up and overwrite the totals.
-Once answered, the acceptance criteria will be:
-- Data Source on the confirmed source: one row per project per expense type (Capex/Opex), Correlation ID = 'ADAPTIVE:' + project id + ':' + expense type.
-- Transform -&gt; cost_plan, coalesce on correlation_id; task = pm_project / dmn_demand via Project Correlation ID.
-- Capex/Opex and category convert in field map scripts (dev confirms field names in the cost_plan dictionary).
-- start_date / end_date = project start / end so ServiceNow builds cost_plan_breakdown; fiscal periods must exist for those dates.
-- Done when pilot project totals equal Adaptive.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Not ready to assign: two answers are needed first, otherwise the dev builds against a guess.&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Where budgets live in Adaptive: project fields or a budget/expense entity (the Discovery output in STRY0067506 lists the candidates).&lt;/li&gt;&lt;li&gt;Cost plans or demand budget totals (STRY0066695) - not both: cost plans roll up and overwrite the totals.&lt;/li&gt;&lt;/ul&gt;
-&lt;p&gt;Once answered, the acceptance criteria will be:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Data Source on the confirmed source: one row per project per expense type (Capex/Opex), Correlation ID = &amp;#x27;ADAPTIVE:&amp;#x27; + project id + &amp;#x27;:&amp;#x27; + expense type.&lt;/li&gt;&lt;li&gt;Transform -&amp;gt; cost_plan, coalesce on correlation_id; task = pm_project / dmn_demand via Project Correlation ID.&lt;/li&gt;&lt;li&gt;Capex/Opex and category convert in field map scripts (dev confirms field names in the cost_plan dictionary).&lt;/li&gt;&lt;li&gt;start_date / end_date = project start / end so ServiceNow builds cost_plan_breakdown; fiscal periods must exist for those dates.&lt;/li&gt;&lt;li&gt;Done when pilot project totals equal Adaptive.&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;On hold until the BA confirms (1) where budgets live in Adaptive and (2) cost plans or demand budget totals (not both).&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -824,13 +710,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="120" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -846,12 +731,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Story</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>What needs correcting</t>
+          <t>Fix</t>
         </is>
       </c>
     </row>
@@ -868,12 +748,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Asana API Connection</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AC 1: no Outbound REST Message record is needed - the Data Source script calls Asana directly and reads the token from property x_mig.asana.token (same as Adaptive). Staging table is u_import_asana_hr_project_portfolio (story says u_imp_asana_hr_portfolio). Project GID = 1208928603143252 (HR Project Portfolio 2026; workspace 5286451799521 is not the project). Use a Data Source 'Custom (Load by Script)' instead of a Scheduled Job, so the transform map runs on the loaded rows: servicenow/asana_data_source.js (MODE 'projects'; MODE 'tasks' for the work plan) already does AC 2-5. Add assignee.name and gid to opt_fields. Token is in property x_mig.asana.token (password2), proven 200 in Dev.</t>
+          <t>Use servicenow/asana_data_source.js in a Data Source instead of a Scheduled Job. No Outbound REST Message needed. Project GID = 1208928603143252. Table = u_import_asana_hr_project_portfolio.</t>
         </is>
       </c>
     </row>
@@ -885,17 +760,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Projects -&gt; pm_project</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Working in Dev. Remaining: (1) scripts for project_manager, u_funding_type, u_sites must return blank on no match (they write 'undefined'); (2) add field map Project Description -&gt; description; (3) Business Sponsor -&gt; u_business_owner (not u_executive_sponsor; Adaptive has no executive sponsor); (4) staging table name is u_import_adaptive_projects; (5) Planned Finish blank -&gt; DueDate? (BA decision).</t>
+          <t>Scripts must leave fields blank when no match (not 'undefined'). Add Project Description -&gt; Detailed Description. Business Sponsor -&gt; Business Owner.</t>
         </is>
       </c>
     </row>
@@ -907,17 +777,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Work Plans -&gt; pm_project_task</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Feed = 'Adaptive Tasks - API' + 'Adaptive Milestones - API' (STRY0067506). Staging needs Correlation ID / Parent Correlation ID / Project Correlation ID. Milestones are a separate Adaptive entity (milestone = true). Run the transform twice (children can arrive before parents). Task state values need BA sign-off.</t>
+          <t>Feed from the Tasks and Milestones Data Sources (STRY0067506). Run the transform twice so every task finds its parent.</t>
         </is>
       </c>
     </row>
@@ -929,17 +794,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Adaptive -&gt; Demands</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Blocked until the Demand vs Project rule exists. 'Upstream pipeline' no longer exists: conversions go in the transform map. Total Budget -&gt; financial_return is wrong (that is expected return). u_executive_sponsor: Adaptive only has Business Sponsor -&gt; u_business_owner.</t>
+          <t>On hold until the Demand vs Project rule is known. Total Budget must not go to financial_return.</t>
         </is>
       </c>
     </row>
@@ -951,17 +811,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Issues -&gt; issue</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Coalesce on correlation_id ("ADAPTIVE:" + issue id) instead of parent + title (titles repeat). Feed = 'Adaptive Issues - API'. Remove 'upstream pipeline' wording; conversions stay in the map. Confirm 'Investigating' exists on issue state.</t>
+          <t>Match records on correlation_id (not parent + title).</t>
         </is>
       </c>
     </row>
@@ -973,17 +828,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Risks -&gt; risk</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Coalesce on correlation_id ("ADAPTIVE:" + risk id) instead of parent + identifier. Feed = 'Adaptive Risks - API'.</t>
+          <t>Match records on correlation_id (not parent + identifier).</t>
         </is>
       </c>
     </row>
@@ -995,17 +845,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Lessons -&gt; u_lessons_learned</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>correlation_id must be "ADAPTIVE:" + id (not the bare /C_PMOLessonsLearned/123), and u_project must look up "ADAPTIVE:" + C_RelatedWorkItem.id - project correlation_ids carry the ADAPTIVE: prefix, so the bare id finds nothing. Feed = 'Adaptive Lessons - API' (does this). Parsing example comment is wrong ('Other' returns 'Other'). Confirm u_lessons_learned has correlation_id.</t>
+          <t>correlation_id and the project lookup must use the "ADAPTIVE:" prefix, or lessons won't find their project.</t>
         </is>
       </c>
     </row>
@@ -1017,17 +862,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Asana -&gt; pm_project</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Switch from CSV to the API feed (STRY0067932). correlation_id = "ASANA:" + gid (gid now available). Only top-level portfolio items are projects; skip Completed/Cancelled. Several mappings conflict with the new HR form (Section -&gt; u_functional_area, Entity -&gt; u_sites, no u_business_category, primary_goal, impacted_business_units): see the 12 questions in mapping/Asana_HR_Project_to_ServiceNow.xlsx.</t>
+          <t>Load from the Asana API, not CSV. Mappings wait on the 12 Asana questions.</t>
         </is>
       </c>
     </row>
@@ -1039,17 +879,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Work in progress</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Asana -&gt; pm_project_task</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Switch to the API feed (asana_data_source.js MODE 'tasks'): Task ID (gid) and Assignee Email now come through, so the earlier blocker is gone. Parent and project come from Parent / Project Correlation ID (not names). Dependency table is planned_task_rel_planned_task.</t>
+          <t>Load from the Asana API (asana_data_source.js, MODE = 'tasks'). Parent comes from Parent Correlation ID, not the task name.</t>
         </is>
       </c>
     </row>
@@ -1064,12 +899,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1083,196 +917,114 @@
           <t>Story</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>STRY0067504</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Connection settings (system properties) in Dev, Test, Prod - no REST Message record</t>
+          <t>STRY0067504 Connection settings</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>STRY0066697 fixes</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Project map fixes, rerun -&gt; 'updated' not 'inserted'</t>
+          <t>STRY0066697 Projects (fix + rerun)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>STRY0067932 / STRY0065263</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Asana portfolio via API</t>
+          <t>STRY0067932 / STRY0065263 Asana projects</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>STRY0067506</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Discovery, then Tasks/Milestones, Risks, Issues, Lessons, Resources, Time Data Sources</t>
+          <t>STRY0067506 Adaptive Data Sources</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>STRY0066699 / STRY0065275</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Work plans (transform twice)</t>
+          <t>STRY0066699 / STRY0065275 Tasks</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>STRY0066701</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Status reports (second map on projects)</t>
+          <t>STRY0066701 Status reports</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>STRY0066718 / STRY0066715 / STRY0067099</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Risks, issues, lessons</t>
+          <t>STRY0066718 / STRY0066715 / STRY0067099 Risks, issues, lessons</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>STRY0066702</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>People and actual effort on tasks</t>
+          <t>STRY0066702 People and hours</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>STRY0066695</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Demands (when rule exists)</t>
+          <t>STRY0066695 Demands (when unblocked)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>STRY0066721</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Cost plans (when decided)</t>
+          <t>STRY0066721 Cost plans (when unblocked)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>STRY0066723</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Attachments - always last</t>
+          <t>STRY0066723 Attachments (last)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Attachments: copy every stored file (no size cap), count found vs copied, update story
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/docs/rm_story_drafts_ready.xlsx
+++ b/docs/rm_story_drafts_ready.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Copy attachments from Asana and Adaptive</t>
+          <t>Copy all attachments from Asana and Adaptive into ServiceNow</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -653,17 +653,17 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>This story is complete when:
-- servicenow/attachments_fix_script.js is run as a Fix Script after all other loads.
-- It is run first with DRY_RUN = true, and the log reviewed. Then it is run with DRY_RUN = false.
-- Files stored in Google Drive, Box, Dropbox or OneDrive are added to the record as a link in a work note.
-- Running it again does not create duplicate files.
-- 10 spot-checked files open correctly in ServiceNow.</t>
+- Every file stored in Asana or Adaptive on a migrated project, task, demand, risk or issue is copied onto the matching ServiceNow record, with the same file name.
+- servicenow/attachments_fix_script.js is run as a Fix Script after all other loads: first with DRY_RUN = true (log reviewed), then with DRY_RUN = false.
+- Links to files kept outside Asana (Google Drive, Box, Dropbox, OneDrive) are added to the record as a work note with the link.
+- The final log line shows copied + skipped = found, and failed = 0. Any failed file is listed and copied by hand.
+- Running it again does not create duplicate files, and 10 spot-checked files open correctly.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>&lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;servicenow/attachments_fix_script.js is run as a Fix Script after all other loads.&lt;/li&gt;&lt;li&gt;It is run first with DRY_RUN = true, and the log reviewed. Then it is run with DRY_RUN = false.&lt;/li&gt;&lt;li&gt;Files stored in Google Drive, Box, Dropbox or OneDrive are added to the record as a link in a work note.&lt;/li&gt;&lt;li&gt;Running it again does not create duplicate files.&lt;/li&gt;&lt;li&gt;10 spot-checked files open correctly in ServiceNow.&lt;/li&gt;&lt;/ul&gt;</t>
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Every file stored in Asana or Adaptive on a migrated project, task, demand, risk or issue is copied onto the matching ServiceNow record, with the same file name.&lt;/li&gt;&lt;li&gt;servicenow/attachments_fix_script.js is run as a Fix Script after all other loads: first with DRY_RUN = true (log reviewed), then with DRY_RUN = false.&lt;/li&gt;&lt;li&gt;Links to files kept outside Asana (Google Drive, Box, Dropbox, OneDrive) are added to the record as a work note with the link.&lt;/li&gt;&lt;li&gt;The final log line shows copied + skipped = found, and failed = 0. Any failed file is listed and copied by hand.&lt;/li&gt;&lt;li&gt;Running it again does not create duplicate files, and 10 spot-checked files open correctly.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>